<commit_message>
bagh dhara bhujel tole
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/nagar bhaipari and estimate misc/jagate chauki bhanjyang/rajan bhujel.xlsx
+++ b/बजेट माग estimate/nagar bhaipari and estimate misc/jagate chauki bhanjyang/rajan bhujel.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{005B6617-EAED-4CCB-A8F9-A3FD4F811B2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11040"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="chauki bhanjyang" sheetId="13" r:id="rId1"/>
@@ -39,7 +40,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'chauki bhanjyang'!$A$1:$K$53</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'chauki bhanjyang'!$1:$8</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -48,6 +49,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -180,22 +183,22 @@
     <t>-13% VAT for aggregates</t>
   </si>
   <si>
-    <t>Project:-Baghdhara pahiro samrakxan</t>
-  </si>
-  <si>
-    <t>Date: 2082/08/08</t>
-  </si>
-  <si>
     <t>Earthwork Excavation in Cutting., Roadway Excavation in all types of Soil by Mechanical  Means ., Road way Excavation in  all types of soil as per Drawing and technical specifications  including  removal of stumps and other deleterious matter, all lifts and lead as per Drawing and instruction of the Engineer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project:-भुजेल टोल बस्ति सडक </t>
+  </si>
+  <si>
+    <t>Date: 2082/09/06</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="13" x14ac:knownFonts="1">
     <font>
@@ -350,9 +353,9 @@
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
@@ -364,7 +367,7 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -388,14 +391,14 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -414,7 +417,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -429,7 +432,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -445,7 +448,25 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -465,32 +486,14 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma 2" xfId="3"/>
+    <cellStyle name="Comma 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2"/>
-    <cellStyle name="Normal 3" xfId="5"/>
-    <cellStyle name="Percent 2" xfId="4"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Normal 3" xfId="5" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Percent 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -506,7 +509,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -600,7 +603,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -659,7 +662,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -723,9 +726,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -763,9 +766,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -800,7 +803,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -835,7 +838,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1008,135 +1011,135 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S53"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" style="19" customWidth="1"/>
-    <col min="2" max="2" width="30.88671875" style="19" customWidth="1"/>
-    <col min="3" max="3" width="4.44140625" style="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.44140625" style="19" customWidth="1"/>
-    <col min="5" max="5" width="8.5546875" style="19" customWidth="1"/>
-    <col min="6" max="6" width="7.33203125" style="19" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" style="19"/>
+    <col min="1" max="1" width="4.7109375" style="19" customWidth="1"/>
+    <col min="2" max="2" width="30.85546875" style="19" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" style="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" style="19" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" style="19" customWidth="1"/>
+    <col min="6" max="6" width="7.28515625" style="19" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="19"/>
     <col min="8" max="8" width="5" style="19" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5546875" style="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.6640625" style="19" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="9.109375" style="19"/>
+    <col min="9" max="9" width="9.5703125" style="19" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="9.140625" style="19"/>
     <col min="13" max="16" width="0" style="19" hidden="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.109375" style="19"/>
+    <col min="17" max="16384" width="9.140625" style="19"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-    </row>
-    <row r="2" spans="1:16" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="47" t="s">
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+    </row>
+    <row r="2" spans="1:16" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A3" s="48" t="s">
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="40"/>
+      <c r="J2" s="40"/>
+      <c r="K2" s="40"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
-      <c r="G3" s="48"/>
-      <c r="H3" s="48"/>
-      <c r="I3" s="48"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="48"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A4" s="48" t="s">
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="41"/>
+      <c r="I3" s="41"/>
+      <c r="J3" s="41"/>
+      <c r="K3" s="41"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="48"/>
-      <c r="I4" s="48"/>
-      <c r="J4" s="48"/>
-      <c r="K4" s="48"/>
-    </row>
-    <row r="5" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A5" s="49" t="s">
+      <c r="B4" s="41"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="41"/>
+      <c r="K4" s="41"/>
+    </row>
+    <row r="5" spans="1:16" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="42" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="49"/>
-      <c r="C5" s="49"/>
-      <c r="D5" s="49"/>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="49"/>
-      <c r="H5" s="49"/>
-      <c r="I5" s="49"/>
-      <c r="J5" s="49"/>
-      <c r="K5" s="49"/>
-    </row>
-    <row r="6" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="44"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="42"/>
+      <c r="I5" s="42"/>
+      <c r="J5" s="42"/>
+      <c r="K5" s="42"/>
+    </row>
+    <row r="6" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="37" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="37"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="37"/>
+      <c r="E6" s="37"/>
+      <c r="F6" s="37"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="45" t="s">
+      <c r="H6" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="45"/>
-      <c r="J6" s="45"/>
-      <c r="K6" s="45"/>
-    </row>
-    <row r="7" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="39" t="s">
+      <c r="I6" s="38"/>
+      <c r="J6" s="38"/>
+      <c r="K6" s="38"/>
+    </row>
+    <row r="7" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="39"/>
-      <c r="C7" s="39"/>
-      <c r="D7" s="39"/>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="45"/>
+      <c r="D7" s="45"/>
+      <c r="E7" s="45"/>
+      <c r="F7" s="45"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="40" t="s">
-        <v>42</v>
-      </c>
-      <c r="I7" s="40"/>
-      <c r="J7" s="40"/>
-      <c r="K7" s="40"/>
-    </row>
-    <row r="8" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="H7" s="46" t="s">
+        <v>43</v>
+      </c>
+      <c r="I7" s="46"/>
+      <c r="J7" s="46"/>
+      <c r="K7" s="46"/>
+    </row>
+    <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
         <v>6</v>
       </c>
@@ -1171,12 +1174,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="171.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" ht="157.5" x14ac:dyDescent="0.25">
       <c r="A9" s="16">
         <v>1</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C9" s="17"/>
       <c r="D9" s="17"/>
@@ -1188,7 +1191,7 @@
       <c r="J9" s="17"/>
       <c r="K9" s="17"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
       <c r="B10" s="32" t="s">
         <v>37</v>
@@ -1229,7 +1232,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="16"/>
       <c r="B11" s="32"/>
       <c r="C11" s="17">
@@ -1259,7 +1262,7 @@
       <c r="O11" s="36"/>
       <c r="P11" s="36"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="16"/>
       <c r="B12" s="32"/>
       <c r="C12" s="17">
@@ -1289,7 +1292,7 @@
       <c r="O12" s="36"/>
       <c r="P12" s="36"/>
     </row>
-    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="34" t="s">
         <v>17</v>
@@ -1314,7 +1317,7 @@
       </c>
       <c r="K13" s="5"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="16"/>
       <c r="B14" s="32" t="s">
         <v>23</v>
@@ -1332,7 +1335,7 @@
       </c>
       <c r="K14" s="17"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="16"/>
       <c r="B15" s="17"/>
       <c r="C15" s="17"/>
@@ -1345,7 +1348,7 @@
       <c r="J15" s="17"/>
       <c r="K15" s="17"/>
     </row>
-    <row r="16" spans="1:16" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" ht="94.5" x14ac:dyDescent="0.25">
       <c r="A16" s="16">
         <v>2</v>
       </c>
@@ -1362,7 +1365,7 @@
       <c r="J16" s="17"/>
       <c r="K16" s="17"/>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="16"/>
       <c r="B17" s="32" t="str">
         <f>B10</f>
@@ -1404,7 +1407,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="16"/>
       <c r="B18" s="32"/>
       <c r="C18" s="17">
@@ -1434,7 +1437,7 @@
       <c r="O18" s="36"/>
       <c r="P18" s="36"/>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="16"/>
       <c r="B19" s="32"/>
       <c r="C19" s="17">
@@ -1464,7 +1467,7 @@
       <c r="O19" s="36"/>
       <c r="P19" s="36"/>
     </row>
-    <row r="20" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="34" t="s">
         <v>17</v>
@@ -1489,7 +1492,7 @@
       </c>
       <c r="K20" s="5"/>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="16"/>
       <c r="B21" s="32" t="s">
         <v>23</v>
@@ -1507,7 +1510,7 @@
       </c>
       <c r="K21" s="17"/>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="16"/>
       <c r="B22" s="17"/>
       <c r="C22" s="17"/>
@@ -1520,7 +1523,7 @@
       <c r="J22" s="17"/>
       <c r="K22" s="17"/>
     </row>
-    <row r="23" spans="1:16" ht="78" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A23" s="16">
         <v>3</v>
       </c>
@@ -1537,7 +1540,7 @@
       <c r="J23" s="17"/>
       <c r="K23" s="17"/>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="16"/>
       <c r="B24" s="32" t="str">
         <f>B17</f>
@@ -1579,7 +1582,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="16"/>
       <c r="B25" s="32"/>
       <c r="C25" s="17">
@@ -1609,7 +1612,7 @@
       <c r="O25" s="36"/>
       <c r="P25" s="36"/>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="16"/>
       <c r="B26" s="32"/>
       <c r="C26" s="17">
@@ -1639,7 +1642,7 @@
       <c r="O26" s="36"/>
       <c r="P26" s="36"/>
     </row>
-    <row r="27" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="34" t="s">
         <v>17</v>
@@ -1664,7 +1667,7 @@
       </c>
       <c r="K27" s="5"/>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="16"/>
       <c r="B28" s="32" t="s">
         <v>31</v>
@@ -1682,7 +1685,7 @@
       </c>
       <c r="K28" s="17"/>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" s="16"/>
       <c r="B29" s="32" t="s">
         <v>32</v>
@@ -1700,7 +1703,7 @@
       </c>
       <c r="K29" s="17"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="16"/>
       <c r="B30" s="32" t="s">
         <v>33</v>
@@ -1718,7 +1721,7 @@
       </c>
       <c r="K30" s="17"/>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="16"/>
       <c r="B31" s="32" t="s">
         <v>34</v>
@@ -1736,7 +1739,7 @@
       </c>
       <c r="K31" s="17"/>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="16"/>
       <c r="B32" s="32" t="s">
         <v>35</v>
@@ -1754,7 +1757,7 @@
       </c>
       <c r="K32" s="17"/>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33" s="16"/>
       <c r="B33" s="17"/>
       <c r="C33" s="17"/>
@@ -1767,7 +1770,7 @@
       <c r="J33" s="17"/>
       <c r="K33" s="17"/>
     </row>
-    <row r="34" spans="1:19" ht="140.4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:19" ht="141.75" x14ac:dyDescent="0.25">
       <c r="A34" s="16">
         <v>4</v>
       </c>
@@ -1784,7 +1787,7 @@
       <c r="J34" s="17"/>
       <c r="K34" s="17"/>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A35" s="16"/>
       <c r="B35" s="32" t="str">
         <f>B24</f>
@@ -1826,7 +1829,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A36" s="16"/>
       <c r="B36" s="32"/>
       <c r="C36" s="17">
@@ -1856,7 +1859,7 @@
       <c r="O36" s="36"/>
       <c r="P36" s="36"/>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A37" s="16"/>
       <c r="B37" s="32"/>
       <c r="C37" s="17">
@@ -1886,7 +1889,7 @@
       <c r="O37" s="36"/>
       <c r="P37" s="36"/>
     </row>
-    <row r="38" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
       <c r="B38" s="34" t="s">
         <v>17</v>
@@ -1911,7 +1914,7 @@
       </c>
       <c r="K38" s="5"/>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A39" s="16"/>
       <c r="B39" s="32" t="s">
         <v>31</v>
@@ -1929,7 +1932,7 @@
       </c>
       <c r="K39" s="17"/>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A40" s="16"/>
       <c r="B40" s="32" t="s">
         <v>32</v>
@@ -1947,7 +1950,7 @@
       </c>
       <c r="K40" s="17"/>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A41" s="16"/>
       <c r="B41" s="32" t="s">
         <v>39</v>
@@ -1965,7 +1968,7 @@
       </c>
       <c r="K41" s="17"/>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="16"/>
       <c r="B42" s="32" t="s">
         <v>40</v>
@@ -1983,7 +1986,7 @@
       </c>
       <c r="K42" s="17"/>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A43" s="16"/>
       <c r="B43" s="17"/>
       <c r="C43" s="17"/>
@@ -1996,7 +1999,7 @@
       <c r="J43" s="17"/>
       <c r="K43" s="17"/>
     </row>
-    <row r="44" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>5</v>
       </c>
@@ -2025,7 +2028,7 @@
       </c>
       <c r="K44" s="5"/>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
       <c r="B45" s="8"/>
       <c r="C45" s="3"/>
@@ -2038,7 +2041,7 @@
       <c r="J45" s="18"/>
       <c r="K45" s="5"/>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A46" s="21"/>
       <c r="B46" s="22" t="s">
         <v>22</v>
@@ -2056,7 +2059,7 @@
       </c>
       <c r="K46" s="25"/>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
       <c r="M47" s="20"/>
       <c r="N47" s="20"/>
       <c r="O47" s="20"/>
@@ -2065,16 +2068,16 @@
       <c r="R47" s="20"/>
       <c r="S47" s="20"/>
     </row>
-    <row r="48" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="26"/>
       <c r="B48" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C48" s="37">
+      <c r="C48" s="43">
         <f>J46</f>
         <v>796238.2567044911</v>
       </c>
-      <c r="D48" s="38"/>
+      <c r="D48" s="44"/>
       <c r="E48" s="9">
         <v>100</v>
       </c>
@@ -2092,79 +2095,72 @@
       <c r="R48" s="19"/>
       <c r="S48" s="19"/>
     </row>
-    <row r="49" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B49" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C49" s="41">
+      <c r="C49" s="47">
         <v>700000</v>
       </c>
-      <c r="D49" s="42"/>
+      <c r="D49" s="48"/>
       <c r="E49" s="9"/>
     </row>
-    <row r="50" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B50" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C50" s="41">
+      <c r="C50" s="47">
         <f>C49-C52-C53</f>
         <v>665000</v>
       </c>
-      <c r="D50" s="42"/>
+      <c r="D50" s="48"/>
       <c r="E50" s="9">
         <f>C50/C48*100</f>
         <v>83.517715256779269</v>
       </c>
     </row>
-    <row r="51" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B51" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="C51" s="43">
+      <c r="C51" s="49">
         <f>C48-C50</f>
         <v>131238.2567044911</v>
       </c>
-      <c r="D51" s="43"/>
+      <c r="D51" s="49"/>
       <c r="E51" s="9">
         <f>100-E50</f>
         <v>16.482284743220731</v>
       </c>
     </row>
-    <row r="52" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B52" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C52" s="37">
+      <c r="C52" s="43">
         <f>C49*0.03</f>
         <v>21000</v>
       </c>
-      <c r="D52" s="38"/>
+      <c r="D52" s="44"/>
       <c r="E52" s="9">
         <v>3</v>
       </c>
     </row>
-    <row r="53" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B53" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C53" s="37">
+      <c r="C53" s="43">
         <f>C49*0.02</f>
         <v>14000</v>
       </c>
-      <c r="D53" s="38"/>
+      <c r="D53" s="44"/>
       <c r="E53" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C52:D52"/>
     <mergeCell ref="C53:D53"/>
     <mergeCell ref="A7:F7"/>
@@ -2173,6 +2169,13 @@
     <mergeCell ref="C49:D49"/>
     <mergeCell ref="C50:D50"/>
     <mergeCell ref="C51:D51"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>

</xml_diff>